<commit_message>
fix: update v0.9.4 score summaries
</commit_message>
<xml_diff>
--- a/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.4-rescored.xlsx
+++ b/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.4-rescored.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="Racd460d422394298"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="Rff027f8efaec432a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1977,7 +1977,7 @@
         <x:v>0.663653</x:v>
       </x:c>
       <x:c r="E25" s="26" t="n">
-        <x:v>0.592258808582866</x:v>
+        <x:v>0.6091200585828661</x:v>
       </x:c>
       <x:c r="F25" s="26" t="str">
         <x:v>平均分</x:v>
@@ -1986,7 +1986,7 @@
         <x:v>0.523549</x:v>
       </x:c>
       <x:c r="H25" s="26" t="n">
-        <x:v>0.4088962386100454</x:v>
+        <x:v>0.42564623861004536</x:v>
       </x:c>
       <x:c r="I25" s="26" t="str">
         <x:v>平均分</x:v>
@@ -1995,7 +1995,7 @@
         <x:v>0.662272</x:v>
       </x:c>
       <x:c r="K25" s="26" t="n">
-        <x:v>0.5306998726822736</x:v>
+        <x:v>0.5599973726822736</x:v>
       </x:c>
       <x:c r="L25" s="26" t="str">
         <x:v>平均分</x:v>
@@ -2004,7 +2004,7 @@
         <x:v>0.515411</x:v>
       </x:c>
       <x:c r="N25" s="47" t="n">
-        <x:v>0.365741058211407</x:v>
+        <x:v>0.3974910582114071</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>